<commit_message>
feat: skip # preamble, parse units row, and report units uniformly across formats
</commit_message>
<xml_diff>
--- a/tests/samples/compliant.xlsx
+++ b/tests/samples/compliant.xlsx
@@ -397,259 +397,351 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T11"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>sample_id</v>
-      </c>
-      <c r="B1" t="str">
-        <v>station_id</v>
-      </c>
-      <c r="C1" t="str">
-        <v>date</v>
-      </c>
-      <c r="D1" t="str">
-        <v>time</v>
-      </c>
-      <c r="E1" t="str">
-        <v>latitude</v>
-      </c>
-      <c r="F1" t="str">
-        <v>longitude</v>
-      </c>
-      <c r="G1" t="str">
-        <v>depth</v>
-      </c>
-      <c r="H1" t="str">
-        <v>depth_flag</v>
-      </c>
-      <c r="I1" t="str">
-        <v>temperature</v>
-      </c>
-      <c r="J1" t="str">
-        <v>temperature_flag</v>
-      </c>
-      <c r="K1" t="str">
-        <v>salinity</v>
-      </c>
-      <c r="L1" t="str">
-        <v>salinity_flag</v>
-      </c>
-      <c r="M1" t="str">
-        <v>dic</v>
-      </c>
-      <c r="N1" t="str">
-        <v>dic_flag</v>
-      </c>
-      <c r="O1" t="str">
-        <v>ta</v>
-      </c>
-      <c r="P1" t="str">
-        <v>ta_flag</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>ph_t_insitu</v>
-      </c>
-      <c r="R1" t="str">
-        <v>ph_t_insitu_flag</v>
-      </c>
-      <c r="S1" t="str">
-        <v>omega_ar</v>
-      </c>
-      <c r="T1" t="str">
-        <v>omega_ar_flag</v>
+        <v># Project ID: OAE-DEMO-01</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>OAE-001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>ST01</v>
-      </c>
-      <c r="C2" t="str">
-        <v>2026-03-14</v>
-      </c>
-      <c r="D2" t="str">
-        <v>09:15:00</v>
-      </c>
-      <c r="E2" t="str">
-        <v>36.8021</v>
-      </c>
-      <c r="F2" t="str">
-        <v>-121.7876</v>
-      </c>
-      <c r="G2" t="str">
-        <v>5.0</v>
-      </c>
-      <c r="H2" t="str">
-        <v>1</v>
-      </c>
-      <c r="I2" t="str">
-        <v>13.42</v>
-      </c>
-      <c r="J2" t="str">
-        <v>1</v>
-      </c>
-      <c r="K2" t="str">
-        <v>33.51</v>
-      </c>
-      <c r="L2" t="str">
-        <v>1</v>
-      </c>
-      <c r="M2" t="str">
-        <v>2045.3</v>
-      </c>
-      <c r="N2" t="str">
-        <v>1</v>
-      </c>
-      <c r="O2" t="str">
-        <v>2231.8</v>
-      </c>
-      <c r="P2" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>8.062</v>
-      </c>
-      <c r="R2" t="str">
-        <v>1</v>
-      </c>
-      <c r="S2" t="str">
-        <v>2.41</v>
-      </c>
-      <c r="T2" t="str">
-        <v>1</v>
+        <v># Experiment ID: OAE-DEMO-01-EXP-A</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>OAE-002</v>
-      </c>
-      <c r="B3" t="str">
-        <v>ST01</v>
-      </c>
-      <c r="C3" t="str">
-        <v>2026-03-14</v>
-      </c>
-      <c r="D3" t="str">
-        <v>09:15:00</v>
-      </c>
-      <c r="E3" t="str">
-        <v>36.8021</v>
-      </c>
-      <c r="F3" t="str">
-        <v>-121.7876</v>
-      </c>
-      <c r="G3" t="str">
-        <v>25.0</v>
-      </c>
-      <c r="H3" t="str">
-        <v>1</v>
-      </c>
-      <c r="I3" t="str">
-        <v>12.10</v>
-      </c>
-      <c r="J3" t="str">
-        <v>1</v>
-      </c>
-      <c r="K3" t="str">
-        <v>33.62</v>
-      </c>
-      <c r="L3" t="str">
-        <v>1</v>
-      </c>
-      <c r="M3" t="str">
-        <v>2078.9</v>
-      </c>
-      <c r="N3" t="str">
-        <v>1</v>
-      </c>
-      <c r="O3" t="str">
-        <v>2240.1</v>
-      </c>
-      <c r="P3" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>8.011</v>
-      </c>
-      <c r="R3" t="str">
-        <v>1</v>
-      </c>
-      <c r="S3" t="str">
-        <v>2.18</v>
-      </c>
-      <c r="T3" t="str">
-        <v>1</v>
+        <v># mCDR experiment type: Alkalinization</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
+        <v># Template version: 1.0.1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v># File last updated on: 2026-03-14</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v># File prepared by: Firstname Lastname (Institution)</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>sample_id</v>
+      </c>
+      <c r="B7" t="str">
+        <v>station_id</v>
+      </c>
+      <c r="C7" t="str">
+        <v>date</v>
+      </c>
+      <c r="D7" t="str">
+        <v>time</v>
+      </c>
+      <c r="E7" t="str">
+        <v>latitude</v>
+      </c>
+      <c r="F7" t="str">
+        <v>longitude</v>
+      </c>
+      <c r="G7" t="str">
+        <v>depth</v>
+      </c>
+      <c r="H7" t="str">
+        <v>depth_flag</v>
+      </c>
+      <c r="I7" t="str">
+        <v>temperature</v>
+      </c>
+      <c r="J7" t="str">
+        <v>temperature_flag</v>
+      </c>
+      <c r="K7" t="str">
+        <v>salinity</v>
+      </c>
+      <c r="L7" t="str">
+        <v>salinity_flag</v>
+      </c>
+      <c r="M7" t="str">
+        <v>dic</v>
+      </c>
+      <c r="N7" t="str">
+        <v>dic_flag</v>
+      </c>
+      <c r="O7" t="str">
+        <v>ta</v>
+      </c>
+      <c r="P7" t="str">
+        <v>ta_flag</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>ph_t_insitu</v>
+      </c>
+      <c r="R7" t="str">
+        <v>ph_t_insitu_flag</v>
+      </c>
+      <c r="S7" t="str">
+        <v>omega_ar</v>
+      </c>
+      <c r="T7" t="str">
+        <v>omega_ar_flag</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="B8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="C8" t="str">
+        <v>YYYY-MM-DD</v>
+      </c>
+      <c r="D8" t="str">
+        <v>hh:mm:ss</v>
+      </c>
+      <c r="E8" t="str">
+        <v>decimal degrees</v>
+      </c>
+      <c r="F8" t="str">
+        <v>decimal degrees</v>
+      </c>
+      <c r="G8" t="str">
+        <v>m</v>
+      </c>
+      <c r="H8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="I8" t="str">
+        <v>deg_C</v>
+      </c>
+      <c r="J8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="K8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="L8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>umol/kg</v>
+      </c>
+      <c r="N8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="O8" t="str">
+        <v>umol/kg</v>
+      </c>
+      <c r="P8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="R8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="S8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="T8" t="str">
+        <v>n.a.</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>OAE-001</v>
+      </c>
+      <c r="B9" t="str">
+        <v>ST01</v>
+      </c>
+      <c r="C9" t="str">
+        <v>2026-03-14</v>
+      </c>
+      <c r="D9" t="str">
+        <v>09:15:00</v>
+      </c>
+      <c r="E9" t="str">
+        <v>36.8021</v>
+      </c>
+      <c r="F9" t="str">
+        <v>-121.7876</v>
+      </c>
+      <c r="G9" t="str">
+        <v>5.0</v>
+      </c>
+      <c r="H9" t="str">
+        <v>1</v>
+      </c>
+      <c r="I9" t="str">
+        <v>13.42</v>
+      </c>
+      <c r="J9" t="str">
+        <v>1</v>
+      </c>
+      <c r="K9" t="str">
+        <v>33.51</v>
+      </c>
+      <c r="L9" t="str">
+        <v>1</v>
+      </c>
+      <c r="M9" t="str">
+        <v>2045.3</v>
+      </c>
+      <c r="N9" t="str">
+        <v>1</v>
+      </c>
+      <c r="O9" t="str">
+        <v>2231.8</v>
+      </c>
+      <c r="P9" t="str">
+        <v>1</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>8.062</v>
+      </c>
+      <c r="R9" t="str">
+        <v>1</v>
+      </c>
+      <c r="S9" t="str">
+        <v>2.41</v>
+      </c>
+      <c r="T9" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>OAE-002</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ST01</v>
+      </c>
+      <c r="C10" t="str">
+        <v>2026-03-14</v>
+      </c>
+      <c r="D10" t="str">
+        <v>09:15:00</v>
+      </c>
+      <c r="E10" t="str">
+        <v>36.8021</v>
+      </c>
+      <c r="F10" t="str">
+        <v>-121.7876</v>
+      </c>
+      <c r="G10" t="str">
+        <v>25.0</v>
+      </c>
+      <c r="H10" t="str">
+        <v>1</v>
+      </c>
+      <c r="I10" t="str">
+        <v>12.10</v>
+      </c>
+      <c r="J10" t="str">
+        <v>1</v>
+      </c>
+      <c r="K10" t="str">
+        <v>33.62</v>
+      </c>
+      <c r="L10" t="str">
+        <v>1</v>
+      </c>
+      <c r="M10" t="str">
+        <v>2078.9</v>
+      </c>
+      <c r="N10" t="str">
+        <v>1</v>
+      </c>
+      <c r="O10" t="str">
+        <v>2240.1</v>
+      </c>
+      <c r="P10" t="str">
+        <v>1</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>8.011</v>
+      </c>
+      <c r="R10" t="str">
+        <v>1</v>
+      </c>
+      <c r="S10" t="str">
+        <v>2.18</v>
+      </c>
+      <c r="T10" t="str">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>OAE-003</v>
       </c>
-      <c r="B4" t="str">
+      <c r="B11" t="str">
         <v>ST02</v>
       </c>
-      <c r="C4" t="str">
+      <c r="C11" t="str">
         <v>2026-03-14</v>
       </c>
-      <c r="D4" t="str">
+      <c r="D11" t="str">
         <v>11:40:00</v>
       </c>
-      <c r="E4" t="str">
+      <c r="E11" t="str">
         <v>36.7955</v>
       </c>
-      <c r="F4" t="str">
+      <c r="F11" t="str">
         <v>-121.8102</v>
       </c>
-      <c r="G4" t="str">
+      <c r="G11" t="str">
         <v>5.0</v>
       </c>
-      <c r="H4" t="str">
-        <v>1</v>
-      </c>
-      <c r="I4" t="str">
+      <c r="H11" t="str">
+        <v>1</v>
+      </c>
+      <c r="I11" t="str">
         <v>13.38</v>
       </c>
-      <c r="J4" t="str">
-        <v>1</v>
-      </c>
-      <c r="K4" t="str">
+      <c r="J11" t="str">
+        <v>1</v>
+      </c>
+      <c r="K11" t="str">
         <v>33.49</v>
       </c>
-      <c r="L4" t="str">
+      <c r="L11" t="str">
         <v>2</v>
       </c>
-      <c r="M4" t="str">
+      <c r="M11" t="str">
         <v>2051.7</v>
       </c>
-      <c r="N4" t="str">
-        <v>1</v>
-      </c>
-      <c r="O4" t="str">
+      <c r="N11" t="str">
+        <v>1</v>
+      </c>
+      <c r="O11" t="str">
         <v>2312.4</v>
       </c>
-      <c r="P4" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q4" t="str">
+      <c r="P11" t="str">
+        <v>1</v>
+      </c>
+      <c r="Q11" t="str">
         <v>8.144</v>
       </c>
-      <c r="R4" t="str">
-        <v>1</v>
-      </c>
-      <c r="S4" t="str">
+      <c r="R11" t="str">
+        <v>1</v>
+      </c>
+      <c r="S11" t="str">
         <v>2.87</v>
       </c>
-      <c r="T4" t="str">
+      <c r="T11" t="str">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:T11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
refactor: derive recommended column names from the protocol templates
</commit_message>
<xml_diff>
--- a/tests/samples/compliant.xlsx
+++ b/tests/samples/compliant.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:T11"/>
+  <dimension ref="A1:R10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -431,64 +431,58 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>sample_id</v>
+        <v>Exp_ID</v>
       </c>
       <c r="B7" t="str">
-        <v>station_id</v>
+        <v>Station_ID</v>
       </c>
       <c r="C7" t="str">
-        <v>date</v>
+        <v>Sample_ID</v>
       </c>
       <c r="D7" t="str">
-        <v>time</v>
+        <v>Year_UTC</v>
       </c>
       <c r="E7" t="str">
-        <v>latitude</v>
+        <v>Month_UTC</v>
       </c>
       <c r="F7" t="str">
-        <v>longitude</v>
+        <v>Day_UTC</v>
       </c>
       <c r="G7" t="str">
-        <v>depth</v>
+        <v>Time_UTC</v>
       </c>
       <c r="H7" t="str">
-        <v>depth_flag</v>
+        <v>Latitude</v>
       </c>
       <c r="I7" t="str">
-        <v>temperature</v>
+        <v>Longitude</v>
       </c>
       <c r="J7" t="str">
-        <v>temperature_flag</v>
+        <v>Depth</v>
       </c>
       <c r="K7" t="str">
-        <v>salinity</v>
+        <v>TEMP_ITS90</v>
       </c>
       <c r="L7" t="str">
-        <v>salinity_flag</v>
+        <v>TEMP_flag</v>
       </c>
       <c r="M7" t="str">
-        <v>dic</v>
+        <v>SAL_PSS78</v>
       </c>
       <c r="N7" t="str">
-        <v>dic_flag</v>
+        <v>SAL_flag</v>
       </c>
       <c r="O7" t="str">
-        <v>ta</v>
+        <v>DIC</v>
       </c>
       <c r="P7" t="str">
-        <v>ta_flag</v>
+        <v>DIC_flag</v>
       </c>
       <c r="Q7" t="str">
-        <v>ph_t_insitu</v>
+        <v>TA</v>
       </c>
       <c r="R7" t="str">
-        <v>ph_t_insitu_flag</v>
-      </c>
-      <c r="S7" t="str">
-        <v>omega_ar</v>
-      </c>
-      <c r="T7" t="str">
-        <v>omega_ar_flag</v>
+        <v>TA_flag</v>
       </c>
     </row>
     <row r="8">
@@ -499,37 +493,37 @@
         <v>n.a.</v>
       </c>
       <c r="C8" t="str">
-        <v>YYYY-MM-DD</v>
+        <v>n.a.</v>
       </c>
       <c r="D8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>n.a.</v>
+      </c>
+      <c r="G8" t="str">
         <v>hh:mm:ss</v>
       </c>
-      <c r="E8" t="str">
+      <c r="H8" t="str">
         <v>decimal degrees</v>
       </c>
-      <c r="F8" t="str">
+      <c r="I8" t="str">
         <v>decimal degrees</v>
       </c>
-      <c r="G8" t="str">
+      <c r="J8" t="str">
         <v>m</v>
       </c>
-      <c r="H8" t="str">
-        <v>n.a.</v>
-      </c>
-      <c r="I8" t="str">
+      <c r="K8" t="str">
         <v>deg_C</v>
       </c>
-      <c r="J8" t="str">
-        <v>n.a.</v>
-      </c>
-      <c r="K8" t="str">
-        <v>n.a.</v>
-      </c>
       <c r="L8" t="str">
         <v>n.a.</v>
       </c>
       <c r="M8" t="str">
-        <v>umol/kg</v>
+        <v>n.a.</v>
       </c>
       <c r="N8" t="str">
         <v>n.a.</v>
@@ -541,207 +535,127 @@
         <v>n.a.</v>
       </c>
       <c r="Q8" t="str">
-        <v>n.a.</v>
+        <v>umol/kg</v>
       </c>
       <c r="R8" t="str">
-        <v>n.a.</v>
-      </c>
-      <c r="S8" t="str">
-        <v>n.a.</v>
-      </c>
-      <c r="T8" t="str">
         <v>n.a.</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>OAE-001</v>
+        <v>OAE-DEMO-01-EXP-A</v>
       </c>
       <c r="B9" t="str">
         <v>ST01</v>
       </c>
       <c r="C9" t="str">
-        <v>2026-03-14</v>
+        <v>10112</v>
       </c>
       <c r="D9" t="str">
+        <v>2026</v>
+      </c>
+      <c r="E9" t="str">
+        <v>3</v>
+      </c>
+      <c r="F9" t="str">
+        <v>14</v>
+      </c>
+      <c r="G9" t="str">
         <v>09:15:00</v>
       </c>
-      <c r="E9" t="str">
+      <c r="H9" t="str">
         <v>36.8021</v>
       </c>
-      <c r="F9" t="str">
+      <c r="I9" t="str">
         <v>-121.7876</v>
       </c>
-      <c r="G9" t="str">
+      <c r="J9" t="str">
         <v>5.0</v>
       </c>
-      <c r="H9" t="str">
-        <v>1</v>
-      </c>
-      <c r="I9" t="str">
+      <c r="K9" t="str">
         <v>13.42</v>
       </c>
-      <c r="J9" t="str">
-        <v>1</v>
-      </c>
-      <c r="K9" t="str">
+      <c r="L9" t="str">
+        <v>2</v>
+      </c>
+      <c r="M9" t="str">
         <v>33.51</v>
       </c>
-      <c r="L9" t="str">
-        <v>1</v>
-      </c>
-      <c r="M9" t="str">
+      <c r="N9" t="str">
+        <v>2</v>
+      </c>
+      <c r="O9" t="str">
         <v>2045.3</v>
       </c>
-      <c r="N9" t="str">
-        <v>1</v>
-      </c>
-      <c r="O9" t="str">
+      <c r="P9" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q9" t="str">
         <v>2231.8</v>
       </c>
-      <c r="P9" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q9" t="str">
-        <v>8.062</v>
-      </c>
       <c r="R9" t="str">
-        <v>1</v>
-      </c>
-      <c r="S9" t="str">
-        <v>2.41</v>
-      </c>
-      <c r="T9" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>OAE-002</v>
+        <v>OAE-DEMO-01-EXP-A</v>
       </c>
       <c r="B10" t="str">
         <v>ST01</v>
       </c>
       <c r="C10" t="str">
-        <v>2026-03-14</v>
+        <v>10113</v>
       </c>
       <c r="D10" t="str">
+        <v>2026</v>
+      </c>
+      <c r="E10" t="str">
+        <v>3</v>
+      </c>
+      <c r="F10" t="str">
+        <v>14</v>
+      </c>
+      <c r="G10" t="str">
         <v>09:15:00</v>
       </c>
-      <c r="E10" t="str">
+      <c r="H10" t="str">
         <v>36.8021</v>
       </c>
-      <c r="F10" t="str">
+      <c r="I10" t="str">
         <v>-121.7876</v>
       </c>
-      <c r="G10" t="str">
+      <c r="J10" t="str">
         <v>25.0</v>
       </c>
-      <c r="H10" t="str">
-        <v>1</v>
-      </c>
-      <c r="I10" t="str">
+      <c r="K10" t="str">
         <v>12.10</v>
       </c>
-      <c r="J10" t="str">
-        <v>1</v>
-      </c>
-      <c r="K10" t="str">
+      <c r="L10" t="str">
+        <v>2</v>
+      </c>
+      <c r="M10" t="str">
         <v>33.62</v>
       </c>
-      <c r="L10" t="str">
-        <v>1</v>
-      </c>
-      <c r="M10" t="str">
+      <c r="N10" t="str">
+        <v>2</v>
+      </c>
+      <c r="O10" t="str">
         <v>2078.9</v>
       </c>
-      <c r="N10" t="str">
-        <v>1</v>
-      </c>
-      <c r="O10" t="str">
+      <c r="P10" t="str">
+        <v>2</v>
+      </c>
+      <c r="Q10" t="str">
         <v>2240.1</v>
       </c>
-      <c r="P10" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q10" t="str">
-        <v>8.011</v>
-      </c>
       <c r="R10" t="str">
-        <v>1</v>
-      </c>
-      <c r="S10" t="str">
-        <v>2.18</v>
-      </c>
-      <c r="T10" t="str">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>OAE-003</v>
-      </c>
-      <c r="B11" t="str">
-        <v>ST02</v>
-      </c>
-      <c r="C11" t="str">
-        <v>2026-03-14</v>
-      </c>
-      <c r="D11" t="str">
-        <v>11:40:00</v>
-      </c>
-      <c r="E11" t="str">
-        <v>36.7955</v>
-      </c>
-      <c r="F11" t="str">
-        <v>-121.8102</v>
-      </c>
-      <c r="G11" t="str">
-        <v>5.0</v>
-      </c>
-      <c r="H11" t="str">
-        <v>1</v>
-      </c>
-      <c r="I11" t="str">
-        <v>13.38</v>
-      </c>
-      <c r="J11" t="str">
-        <v>1</v>
-      </c>
-      <c r="K11" t="str">
-        <v>33.49</v>
-      </c>
-      <c r="L11" t="str">
-        <v>2</v>
-      </c>
-      <c r="M11" t="str">
-        <v>2051.7</v>
-      </c>
-      <c r="N11" t="str">
-        <v>1</v>
-      </c>
-      <c r="O11" t="str">
-        <v>2312.4</v>
-      </c>
-      <c r="P11" t="str">
-        <v>1</v>
-      </c>
-      <c r="Q11" t="str">
-        <v>8.144</v>
-      </c>
-      <c r="R11" t="str">
-        <v>1</v>
-      </c>
-      <c r="S11" t="str">
-        <v>2.87</v>
-      </c>
-      <c r="T11" t="str">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:T11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:R10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>